<commit_message>
fix(timeseries): updated codebase from timeseries repo & added run docs in readme
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P3_2stages_VRU.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P3_2stages_VRU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wmollel\Documents\MEET2\input\Studies\C3\C3_Prototypical_Sites\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kayarn/sources/xpower/csu/MAES/input/Studies/C3/C3_Prototypical_Sites/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7974B0F-B94D-40C9-9D70-843A4CEC99C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13B2559-9DED-4B4B-BC1F-962A7541722E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="925" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4480" yWindow="500" windowWidth="31360" windowHeight="21900" tabRatio="925" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -1407,13 +1407,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1429,25 +1429,25 @@
         <v>365</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>205</v>
       </c>
@@ -1464,12 +1464,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>160</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>96</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1533,7 +1533,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>41</v>
       </c>
@@ -1549,16 +1549,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" customWidth="1"/>
     <col min="4" max="4" width="64" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="12" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>4</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -1600,14 +1600,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2690304-5371-4DEF-8D7E-371EB1C22F96}">
   <dimension ref="A1:S9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="63.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="63.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="20" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="20" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
         <v>4</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>100</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>100</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>100</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>100</v>
       </c>
@@ -2146,17 +2146,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="13" width="15.7109375" style="4" customWidth="1"/>
-    <col min="14" max="14" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" customWidth="1"/>
-    <col min="17" max="17" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="13" width="15.6640625" style="4" customWidth="1"/>
+    <col min="14" max="14" width="24.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="47.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.6640625" customWidth="1"/>
+    <col min="17" max="17" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="3" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
         <v>4</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -2256,7 +2256,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -2356,7 +2356,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>100</v>
       </c>
@@ -2456,7 +2456,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>100</v>
       </c>
@@ -2506,7 +2506,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>100</v>
       </c>
@@ -2556,7 +2556,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>100</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="F10"/>
       <c r="G10"/>
       <c r="H10"/>
@@ -2616,7 +2616,7 @@
       <c r="L10"/>
       <c r="M10"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>100</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>100</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>100</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>100</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>100</v>
       </c>
@@ -2866,7 +2866,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>100</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>100</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>100</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="F19"/>
       <c r="G19"/>
       <c r="H19"/>
@@ -3033,26 +3033,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:U16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="12" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="12" width="26.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="12" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="12" customFormat="1" ht="80" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>4</v>
       </c>
@@ -3117,7 +3117,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -3182,34 +3182,34 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F7"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F8"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F9"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F10"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F11"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F12"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F13"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F14"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F15"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="F16"/>
     </row>
   </sheetData>
@@ -3221,42 +3221,40 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:AF3"/>
-  <sheetFormatPr defaultColWidth="66.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="66.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.5" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="63.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="63.6640625" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="12" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="12" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>4</v>
       </c>
@@ -3354,7 +3352,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -3452,7 +3450,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -3559,58 +3557,58 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:BB9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" customWidth="1"/>
+    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.5" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="15" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="11" bestFit="1" customWidth="1"/>
-    <col min="33" max="34" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.5" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="10" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="9.5" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="15" customWidth="1"/>
-    <col min="40" max="41" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="40" max="41" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="10" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="45" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="17.5" bestFit="1" customWidth="1"/>
     <col min="48" max="49" width="15" bestFit="1" customWidth="1"/>
     <col min="50" max="50" width="14" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="16" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="47.1640625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" s="18" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:54" s="18" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
         <v>4</v>
       </c>
@@ -3774,7 +3772,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -3937,7 +3935,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="3" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -4100,7 +4098,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="4" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -4263,7 +4261,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="5" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -4426,7 +4424,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="6" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>100</v>
       </c>
@@ -4589,7 +4587,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>100</v>
       </c>
@@ -4752,7 +4750,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="8" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>100</v>
       </c>
@@ -4915,7 +4913,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:54" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>100</v>
       </c>
@@ -5088,18 +5086,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A904CBC9-E240-4A6F-BB4B-8DAB1536C2C9}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="47.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="80" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
         <v>4</v>
       </c>
@@ -5158,7 +5156,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -5217,7 +5215,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -5285,18 +5283,18 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09131FE7-5CF0-4155-B869-9951A97BC4D6}">
   <dimension ref="A1:G130"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -5319,7 +5317,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>67</v>
       </c>
@@ -5340,7 +5338,7 @@
       </c>
       <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>67</v>
       </c>
@@ -5360,7 +5358,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>67</v>
       </c>
@@ -5380,7 +5378,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>67</v>
       </c>
@@ -5400,7 +5398,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>67</v>
       </c>
@@ -5420,7 +5418,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>67</v>
       </c>
@@ -5440,7 +5438,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>67</v>
       </c>
@@ -5460,7 +5458,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>67</v>
       </c>
@@ -5480,7 +5478,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>67</v>
       </c>
@@ -5500,7 +5498,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>67</v>
       </c>
@@ -5520,7 +5518,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -5540,7 +5538,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>67</v>
       </c>
@@ -5560,7 +5558,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -5580,7 +5578,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -5600,7 +5598,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -5620,7 +5618,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>67</v>
       </c>
@@ -5640,7 +5638,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>67</v>
       </c>
@@ -5663,7 +5661,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>67</v>
       </c>
@@ -5686,7 +5684,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>67</v>
       </c>
@@ -5709,7 +5707,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -5732,7 +5730,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -5755,7 +5753,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>67</v>
       </c>
@@ -5778,7 +5776,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -5801,7 +5799,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -5824,7 +5822,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>67</v>
       </c>
@@ -5847,7 +5845,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>67</v>
       </c>
@@ -5870,7 +5868,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>67</v>
       </c>
@@ -5893,7 +5891,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>67</v>
       </c>
@@ -5916,7 +5914,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>67</v>
       </c>
@@ -5939,7 +5937,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -5962,7 +5960,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -5985,7 +5983,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -6008,7 +6006,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>67</v>
       </c>
@@ -6031,7 +6029,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>67</v>
       </c>
@@ -6054,7 +6052,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>67</v>
       </c>
@@ -6077,7 +6075,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>67</v>
       </c>
@@ -6100,7 +6098,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>67</v>
       </c>
@@ -6123,7 +6121,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -6146,7 +6144,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>67</v>
       </c>
@@ -6169,7 +6167,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>67</v>
       </c>
@@ -6192,7 +6190,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>67</v>
       </c>
@@ -6215,7 +6213,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>67</v>
       </c>
@@ -6238,7 +6236,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>67</v>
       </c>
@@ -6261,7 +6259,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>67</v>
       </c>
@@ -6284,7 +6282,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>67</v>
       </c>
@@ -6307,7 +6305,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>67</v>
       </c>
@@ -6330,7 +6328,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>67</v>
       </c>
@@ -6353,7 +6351,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>67</v>
       </c>
@@ -6376,7 +6374,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>67</v>
       </c>
@@ -6399,7 +6397,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>67</v>
       </c>
@@ -6422,7 +6420,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>67</v>
       </c>
@@ -6445,7 +6443,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>67</v>
       </c>
@@ -6468,7 +6466,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>67</v>
       </c>
@@ -6491,7 +6489,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>67</v>
       </c>
@@ -6514,7 +6512,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>67</v>
       </c>
@@ -6537,7 +6535,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>67</v>
       </c>
@@ -6560,7 +6558,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -6583,7 +6581,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -6606,7 +6604,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -6629,7 +6627,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>67</v>
       </c>
@@ -6652,7 +6650,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>67</v>
       </c>
@@ -6675,7 +6673,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>67</v>
       </c>
@@ -6698,7 +6696,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>67</v>
       </c>
@@ -6721,7 +6719,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -6744,7 +6742,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>67</v>
       </c>
@@ -6767,7 +6765,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>67</v>
       </c>
@@ -6790,7 +6788,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>67</v>
       </c>
@@ -6813,7 +6811,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>67</v>
       </c>
@@ -6836,7 +6834,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>67</v>
       </c>
@@ -6859,7 +6857,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>67</v>
       </c>
@@ -6882,7 +6880,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>67</v>
       </c>
@@ -6905,7 +6903,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>67</v>
       </c>
@@ -6928,7 +6926,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>67</v>
       </c>
@@ -6951,7 +6949,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>67</v>
       </c>
@@ -6974,7 +6972,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>67</v>
       </c>
@@ -6997,7 +6995,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>67</v>
       </c>
@@ -7020,7 +7018,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>67</v>
       </c>
@@ -7043,7 +7041,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>67</v>
       </c>
@@ -7066,7 +7064,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>67</v>
       </c>
@@ -7089,7 +7087,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>67</v>
       </c>
@@ -7112,7 +7110,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>67</v>
       </c>
@@ -7135,7 +7133,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>67</v>
       </c>
@@ -7158,7 +7156,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>67</v>
       </c>
@@ -7181,7 +7179,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>67</v>
       </c>
@@ -7204,7 +7202,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>67</v>
       </c>
@@ -7227,7 +7225,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>67</v>
       </c>
@@ -7250,7 +7248,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>67</v>
       </c>
@@ -7273,7 +7271,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>67</v>
       </c>
@@ -7296,7 +7294,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>67</v>
       </c>
@@ -7319,7 +7317,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>67</v>
       </c>
@@ -7342,7 +7340,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>67</v>
       </c>
@@ -7365,7 +7363,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>67</v>
       </c>
@@ -7388,7 +7386,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>67</v>
       </c>
@@ -7411,7 +7409,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>67</v>
       </c>
@@ -7434,7 +7432,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>67</v>
       </c>
@@ -7457,7 +7455,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>67</v>
       </c>
@@ -7480,7 +7478,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>67</v>
       </c>
@@ -7503,7 +7501,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>67</v>
       </c>
@@ -7526,7 +7524,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>67</v>
       </c>
@@ -7549,7 +7547,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>67</v>
       </c>
@@ -7572,7 +7570,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>67</v>
       </c>
@@ -7595,7 +7593,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>67</v>
       </c>
@@ -7618,7 +7616,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>67</v>
       </c>
@@ -7641,7 +7639,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>67</v>
       </c>
@@ -7664,7 +7662,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>67</v>
       </c>
@@ -7687,7 +7685,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>67</v>
       </c>
@@ -7710,7 +7708,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>67</v>
       </c>
@@ -7733,7 +7731,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>67</v>
       </c>
@@ -7756,7 +7754,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>67</v>
       </c>
@@ -7779,7 +7777,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>67</v>
       </c>
@@ -7802,7 +7800,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>67</v>
       </c>
@@ -7825,7 +7823,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>67</v>
       </c>
@@ -7848,7 +7846,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>67</v>
       </c>
@@ -7871,7 +7869,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>67</v>
       </c>
@@ -7894,7 +7892,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>67</v>
       </c>
@@ -7917,7 +7915,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>67</v>
       </c>
@@ -7940,7 +7938,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>67</v>
       </c>
@@ -7963,7 +7961,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>67</v>
       </c>
@@ -7986,7 +7984,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>67</v>
       </c>
@@ -8009,7 +8007,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>67</v>
       </c>
@@ -8032,7 +8030,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>67</v>
       </c>
@@ -8055,7 +8053,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>67</v>
       </c>
@@ -8078,7 +8076,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>67</v>
       </c>

</xml_diff>